<commit_message>
altera raw bias para absolute error e no percentual bias - relative error
</commit_message>
<xml_diff>
--- a/artigo/tabel_TFR.xlsx
+++ b/artigo/tabel_TFR.xlsx
@@ -2202,7 +2202,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2227,7 +2227,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2277,7 +2277,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2352,7 +2352,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2427,7 +2427,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2477,7 +2477,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2502,7 +2502,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2552,7 +2552,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2602,7 +2602,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2652,7 +2652,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2702,7 +2702,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2727,7 +2727,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2752,7 +2752,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2802,7 +2802,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2827,7 +2827,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2852,7 +2852,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2877,7 +2877,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2902,7 +2902,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2927,7 +2927,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3002,7 +3002,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3027,7 +3027,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3077,7 +3077,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3102,7 +3102,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3127,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3227,7 +3227,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3252,7 +3252,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3302,7 +3302,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3352,7 +3352,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3402,7 +3402,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3427,7 +3427,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3477,7 +3477,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3627,7 +3627,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3652,7 +3652,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3677,7 +3677,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3702,7 +3702,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3727,7 +3727,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3752,7 +3752,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3777,7 +3777,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3802,7 +3802,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3827,7 +3827,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3852,7 +3852,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3877,7 +3877,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3902,7 +3902,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3952,7 +3952,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -3977,7 +3977,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Raw bias</t>
+          <t>Absolute error</t>
         </is>
       </c>
     </row>
@@ -4002,7 +4002,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4027,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4077,7 +4077,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4102,7 +4102,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4127,7 +4127,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4152,7 +4152,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4177,7 +4177,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4202,7 +4202,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4227,7 +4227,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4277,7 +4277,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4327,7 +4327,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4427,7 +4427,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4452,7 +4452,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4477,7 +4477,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4502,7 +4502,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4527,7 +4527,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4552,7 +4552,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4577,7 +4577,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4602,7 +4602,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4652,7 +4652,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4677,7 +4677,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4702,7 +4702,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4752,7 +4752,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4777,7 +4777,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4802,7 +4802,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4827,7 +4827,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4852,7 +4852,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4877,7 +4877,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4927,7 +4927,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4952,7 +4952,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -4977,7 +4977,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5027,7 +5027,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5052,7 +5052,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5077,7 +5077,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5102,7 +5102,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5127,7 +5127,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5177,7 +5177,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5202,7 +5202,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5227,7 +5227,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5252,7 +5252,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5277,7 +5277,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5327,7 +5327,7 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5352,7 +5352,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5377,7 +5377,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5402,7 +5402,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5452,7 +5452,7 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5477,7 +5477,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5527,7 +5527,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5552,7 +5552,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5577,7 +5577,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5602,7 +5602,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5627,7 +5627,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5652,7 +5652,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5677,7 +5677,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5702,7 +5702,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5727,7 +5727,7 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5752,7 +5752,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>
@@ -5777,7 +5777,7 @@
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Percent bias</t>
+          <t>Relative error</t>
         </is>
       </c>
     </row>

</xml_diff>